<commit_message>
Updated excel data set and added processing file
I slightly reformatted my excel data collection layout and updated it by adding the latest data. Alongside, I added a folder in which my processing sketch will be updated and worked on.
</commit_message>
<xml_diff>
--- a/Recorded Data for DD.xlsx
+++ b/Recorded Data for DD.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\dearData_100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F103FE24-90F7-41CF-869A-4C902B67998F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46FAEFDA-3BC7-4AAD-A7BF-56BB3F38ABAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D9342B3C-2640-4AC7-BBCB-770C99F77758}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$2:$F$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,22 +42,62 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="15">
   <si>
-    <t>Dear Data Project</t>
+    <t>Amount</t>
   </si>
   <si>
-    <t>yo</t>
+    <t>Category</t>
   </si>
   <si>
-    <t>why is it 2</t>
+    <t>Need/Want</t>
+  </si>
+  <si>
+    <t>Categories:</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Shopping</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Dear Data Project (data set on spending)</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Need</t>
+  </si>
+  <si>
+    <t>Want</t>
+  </si>
+  <si>
+    <t>Data Points:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$£-809]* #,##0.00_-;\-[$£-809]* #,##0.00_-;_-[$£-809]* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,13 +105,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -80,16 +154,45 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -422,31 +525,1121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61FBEC59-24E1-403E-B479-945543868AF5}">
-  <dimension ref="B2:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:I202"/>
+  <sheetFormatPr defaultColWidth="13.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" style="1"/>
+    <col min="2" max="2" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" style="1"/>
+    <col min="8" max="8" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="13.6640625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="4">
+        <f>COUNT(B:B)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+      <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+      <c r="F3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.2902777777777778</v>
+      </c>
+      <c r="D4" s="7">
+        <v>7.5</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B5" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.30416666666666664</v>
+      </c>
+      <c r="D5" s="7">
+        <v>34.950000000000003</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.37777777777777777</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2.7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.52638888888888891</v>
+      </c>
+      <c r="D7" s="7">
+        <v>4</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.53472222222222221</v>
+      </c>
+      <c r="D8" s="7">
+        <v>1.75</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="5">
+        <v>46314</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.58888888888888891</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1.85</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C10" s="6">
+        <v>9.6527777777777782E-2</v>
+      </c>
+      <c r="D10" s="7">
+        <v>12.8</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B11" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D11" s="7">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.58125000000000004</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1.85</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.72986111111111107</v>
+      </c>
+      <c r="D13" s="7">
+        <v>1.7</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.74722222222222223</v>
+      </c>
+      <c r="D14" s="7">
+        <v>39.99</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" s="5">
+        <v>46315</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.76458333333333328</v>
+      </c>
+      <c r="D15" s="7">
+        <v>34.76</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B16" s="5">
+        <v>46316</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.42083333333333334</v>
+      </c>
+      <c r="D16" s="7">
+        <v>11.9</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="5">
+        <v>46317</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="7">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="5">
+        <v>46318</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.62638888888888888</v>
+      </c>
+      <c r="D18" s="7">
+        <v>4</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="5">
+        <v>46318</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.62708333333333333</v>
+      </c>
+      <c r="D19" s="7">
+        <v>1.65</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="5">
+        <v>46319</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.10277777777777777</v>
+      </c>
+      <c r="D20" s="7">
+        <v>12.8</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="5">
+        <v>46319</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.15138888888888888</v>
+      </c>
+      <c r="D21" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="5">
+        <v>46320</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="8">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="D23" s="8">
+        <v>6.55</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.4597222222222222</v>
+      </c>
+      <c r="D24" s="8">
+        <v>7.63</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="D25" s="8">
+        <v>4.6900000000000004</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.68194444444444446</v>
+      </c>
+      <c r="D26" s="8">
+        <v>8.59</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0.72986111111111107</v>
+      </c>
+      <c r="D27" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C28" s="6">
+        <v>0.74027777777777781</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C29" s="6">
+        <v>0.12152777777777778</v>
+      </c>
+      <c r="D29" s="8">
+        <v>6.55</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C30" s="6">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="D30" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C31" s="6">
+        <v>0.37361111111111112</v>
+      </c>
+      <c r="D31" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B32" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C32" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D32" s="8">
+        <v>4.74</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C33" s="6">
+        <v>0.50555555555555554</v>
+      </c>
+      <c r="D33" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C34" s="6">
+        <v>0.5854166666666667</v>
+      </c>
+      <c r="D34" s="8">
+        <v>5.99</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C35" s="6">
+        <v>0.65902777777777777</v>
+      </c>
+      <c r="D35" s="8">
+        <v>5</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B36" s="9">
+        <v>46323</v>
+      </c>
+      <c r="D36" s="10"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D37" s="10"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D38" s="10"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D39" s="10"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D40" s="10"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D41" s="10"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D42" s="10"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D43" s="10"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D44" s="10"/>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D45" s="10"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D46" s="10"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D47" s="10"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D48" s="10"/>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D49" s="10"/>
+    </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D50" s="10"/>
+    </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D51" s="10"/>
+    </row>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D52" s="10"/>
+    </row>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D53" s="10"/>
+    </row>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D54" s="10"/>
+    </row>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D55" s="10"/>
+    </row>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D56" s="10"/>
+    </row>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D57" s="10"/>
+    </row>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D58" s="10"/>
+    </row>
+    <row r="59" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D59" s="10"/>
+    </row>
+    <row r="60" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D60" s="10"/>
+    </row>
+    <row r="61" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D61" s="10"/>
+    </row>
+    <row r="62" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D62" s="10"/>
+    </row>
+    <row r="63" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D63" s="10"/>
+    </row>
+    <row r="64" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D64" s="10"/>
+    </row>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D65" s="10"/>
+    </row>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D66" s="10"/>
+    </row>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D67" s="10"/>
+    </row>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D68" s="10"/>
+    </row>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D69" s="10"/>
+    </row>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D70" s="10"/>
+    </row>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D71" s="10"/>
+    </row>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D72" s="10"/>
+    </row>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D73" s="10"/>
+    </row>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D74" s="10"/>
+    </row>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D75" s="10"/>
+    </row>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D76" s="10"/>
+    </row>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D77" s="10"/>
+    </row>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D78" s="10"/>
+    </row>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D79" s="10"/>
+    </row>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D80" s="10"/>
+    </row>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D81" s="10"/>
+    </row>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D82" s="10"/>
+    </row>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D83" s="10"/>
+    </row>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D84" s="10"/>
+    </row>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D85" s="10"/>
+    </row>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D86" s="10"/>
+    </row>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D87" s="10"/>
+    </row>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D88" s="10"/>
+    </row>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D89" s="10"/>
+    </row>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D90" s="10"/>
+    </row>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D91" s="10"/>
+    </row>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D92" s="10"/>
+    </row>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D93" s="10"/>
+    </row>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D94" s="10"/>
+    </row>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D95" s="10"/>
+    </row>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D96" s="10"/>
+    </row>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D97" s="10"/>
+    </row>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D98" s="10"/>
+    </row>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D99" s="10"/>
+    </row>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D100" s="10"/>
+    </row>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D101" s="10"/>
+    </row>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D102" s="10"/>
+    </row>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D103" s="10"/>
+    </row>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D104" s="10"/>
+    </row>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D105" s="10"/>
+    </row>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D106" s="10"/>
+    </row>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D107" s="10"/>
+    </row>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D108" s="10"/>
+    </row>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D109" s="10"/>
+    </row>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D110" s="10"/>
+    </row>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D111" s="10"/>
+    </row>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D112" s="10"/>
+    </row>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D113" s="10"/>
+    </row>
+    <row r="114" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D114" s="10"/>
+    </row>
+    <row r="115" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D115" s="10"/>
+    </row>
+    <row r="116" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D116" s="10"/>
+    </row>
+    <row r="117" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D117" s="10"/>
+    </row>
+    <row r="118" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D118" s="10"/>
+    </row>
+    <row r="119" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D119" s="10"/>
+    </row>
+    <row r="120" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D120" s="10"/>
+    </row>
+    <row r="121" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D121" s="10"/>
+    </row>
+    <row r="122" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D122" s="10"/>
+    </row>
+    <row r="123" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D123" s="10"/>
+    </row>
+    <row r="124" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D124" s="10"/>
+    </row>
+    <row r="125" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D125" s="10"/>
+    </row>
+    <row r="126" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D126" s="10"/>
+    </row>
+    <row r="127" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D127" s="10"/>
+    </row>
+    <row r="128" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D128" s="10"/>
+    </row>
+    <row r="129" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D129" s="10"/>
+    </row>
+    <row r="130" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D130" s="10"/>
+    </row>
+    <row r="131" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D131" s="10"/>
+    </row>
+    <row r="132" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D132" s="10"/>
+    </row>
+    <row r="133" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D133" s="10"/>
+    </row>
+    <row r="134" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D134" s="10"/>
+    </row>
+    <row r="135" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D135" s="10"/>
+    </row>
+    <row r="136" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D136" s="10"/>
+    </row>
+    <row r="137" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D137" s="10"/>
+    </row>
+    <row r="138" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D138" s="10"/>
+    </row>
+    <row r="139" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D139" s="10"/>
+    </row>
+    <row r="140" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D140" s="10"/>
+    </row>
+    <row r="141" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D141" s="10"/>
+    </row>
+    <row r="142" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D142" s="10"/>
+    </row>
+    <row r="143" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D143" s="10"/>
+    </row>
+    <row r="144" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D144" s="10"/>
+    </row>
+    <row r="145" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D145" s="10"/>
+    </row>
+    <row r="146" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D146" s="10"/>
+    </row>
+    <row r="147" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D147" s="10"/>
+    </row>
+    <row r="148" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D148" s="10"/>
+    </row>
+    <row r="149" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D149" s="10"/>
+    </row>
+    <row r="150" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D150" s="10"/>
+    </row>
+    <row r="151" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D151" s="10"/>
+    </row>
+    <row r="152" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D152" s="10"/>
+    </row>
+    <row r="153" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D153" s="10"/>
+    </row>
+    <row r="154" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D154" s="10"/>
+    </row>
+    <row r="155" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D155" s="10"/>
+    </row>
+    <row r="156" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D156" s="10"/>
+    </row>
+    <row r="157" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D157" s="10"/>
+    </row>
+    <row r="158" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D158" s="10"/>
+    </row>
+    <row r="159" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D159" s="10"/>
+    </row>
+    <row r="160" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D160" s="10"/>
+    </row>
+    <row r="161" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D161" s="10"/>
+    </row>
+    <row r="162" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D162" s="10"/>
+    </row>
+    <row r="163" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D163" s="10"/>
+    </row>
+    <row r="164" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D164" s="10"/>
+    </row>
+    <row r="165" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D165" s="10"/>
+    </row>
+    <row r="166" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D166" s="10"/>
+    </row>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D167" s="10"/>
+    </row>
+    <row r="168" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D168" s="10"/>
+    </row>
+    <row r="169" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D169" s="10"/>
+    </row>
+    <row r="170" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D170" s="10"/>
+    </row>
+    <row r="171" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D171" s="10"/>
+    </row>
+    <row r="172" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D172" s="10"/>
+    </row>
+    <row r="173" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D173" s="10"/>
+    </row>
+    <row r="174" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D174" s="10"/>
+    </row>
+    <row r="175" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D175" s="10"/>
+    </row>
+    <row r="176" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D176" s="10"/>
+    </row>
+    <row r="177" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D177" s="10"/>
+    </row>
+    <row r="178" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D178" s="10"/>
+    </row>
+    <row r="179" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D179" s="10"/>
+    </row>
+    <row r="180" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D180" s="10"/>
+    </row>
+    <row r="181" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D181" s="10"/>
+    </row>
+    <row r="182" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D182" s="10"/>
+    </row>
+    <row r="183" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D183" s="10"/>
+    </row>
+    <row r="184" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D184" s="10"/>
+    </row>
+    <row r="185" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D185" s="10"/>
+    </row>
+    <row r="186" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D186" s="10"/>
+    </row>
+    <row r="187" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D187" s="10"/>
+    </row>
+    <row r="188" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D188" s="10"/>
+    </row>
+    <row r="189" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D189" s="10"/>
+    </row>
+    <row r="190" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D190" s="10"/>
+    </row>
+    <row r="191" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D191" s="10"/>
+    </row>
+    <row r="192" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D192" s="10"/>
+    </row>
+    <row r="193" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D193" s="10"/>
+    </row>
+    <row r="194" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D194" s="10"/>
+    </row>
+    <row r="195" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D195" s="10"/>
+    </row>
+    <row r="196" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D196" s="10"/>
+    </row>
+    <row r="197" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D197" s="10"/>
+    </row>
+    <row r="198" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D198" s="10"/>
+    </row>
+    <row r="199" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D199" s="10"/>
+    </row>
+    <row r="200" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D200" s="10"/>
+    </row>
+    <row r="201" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D201" s="10"/>
+    </row>
+    <row r="202" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D202" s="10"/>
+    </row>
   </sheetData>
+  <autoFilter ref="B2:F5" xr:uid="{61FBEC59-24E1-403E-B479-945543868AF5}">
+    <filterColumn colId="0" showButton="0"/>
+    <filterColumn colId="1" showButton="0"/>
+    <filterColumn colId="2" showButton="0"/>
+    <filterColumn colId="3" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
-    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -621,15 +1814,15 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17F07A12-5357-4212-A6CB-979F8303843A}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="a59ad716-875e-46ef-9311-f1d20923e9b6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>